<commit_message>
Corrige les liens cassés, l'incohérence de navigation et nettoie le dépôt
- Retire le bouton "Modalités d'épreuve" devenu inutile sur la page Réalisations
- Corrige l'affichage en colonne désorganisée des notices 1ère/2ème année (icône alignée en haut, texte dans un span)
- Renomme DHCP-failover.docx en DHCP failover.docx et met à jour les références
- Corrige le lien vers la fiche mémo Site Tracker (nom de fichier exact)
- Ajoute le lien Contact manquant dans la nav de la page d'accueil
- Retire desktop.ini du suivi git et ajoute un .gitignore (fichiers système Windows, verrous Office)
- Supprime ~30 Mo de fichiers obsolètes et jamais référencés sur le site (vidéos, captures et documents orphelins)
</commit_message>
<xml_diff>
--- a/Tableau de synthèse Esra (1).xlsx
+++ b/Tableau de synthèse Esra (1).xlsx
@@ -1,29 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eatia\Desktop\PortfolioNew\portfolio\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41F19D72-4247-48B4-8C0A-715EE7E0D634}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F25F18B-816E-47E6-8F6A-353296643EDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tableau de synthèse Épreuve E4" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Tableau de synthèse Épreuve E4'!$A$1:$H$95</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Tableau de synthèse Épreuve E4'!$A$1:$H$97</definedName>
   </definedNames>
   <calcPr calcId="101716"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="104">
   <si>
     <t>Gérer le patrimoine informatique</t>
   </si>
@@ -116,9 +116,6 @@
     <t>Centre de formation : EFREI Villejuif</t>
   </si>
   <si>
-    <t>C1 - Recensement du parc informatique (matériel, VMs, logiciels, câblage) via GLPI</t>
-  </si>
-  <si>
     <t>C1 - Inventaire complet du matériel virtuel/réel, cartographie du réseau, listage des logiciels</t>
   </si>
   <si>
@@ -137,18 +134,12 @@
     <t>C2 - TP complet sur ITIL et ISO 27001 (analyse non-conformités, rédaction procédures)</t>
   </si>
   <si>
-    <t>C2 - Préparation réunion RH pour mise en conformité RGPD de Sitetracker</t>
-  </si>
-  <si>
     <t>C3 - TP Active Directory (création comptes, groupes, droits, moindre privilège)</t>
   </si>
   <si>
     <t>C3 - Vérification que seul l'administrateur a les droits administrateur</t>
   </si>
   <si>
-    <t>C3 - Définition de 15 profils utilisateurs sur Sitetracker pour +70 utilisateurs</t>
-  </si>
-  <si>
     <t>C3 - Attribution des droits et accès selon licence et profil (employés, négociateurs, API)</t>
   </si>
   <si>
@@ -191,18 +182,12 @@
     <t>TP HAProxy (load balancing, terminaison SSL)</t>
   </si>
   <si>
-    <t>TP Suricata (IDS/IPS)</t>
-  </si>
-  <si>
     <t>TP Snort (IDS/IPS)</t>
   </si>
   <si>
     <t>TP pfSense (firewall, règles de filtrage)</t>
   </si>
   <si>
-    <t>TP Zabbix (supervision)</t>
-  </si>
-  <si>
     <t>TP Nagios (supervision)</t>
   </si>
   <si>
@@ -215,15 +200,9 @@
     <t>TP GLPI : définition des catégories ITIL, règles d'affectation automatique</t>
   </si>
   <si>
-    <t>Utilisation de l'outil de ticketing Salesforce</t>
-  </si>
-  <si>
     <t>Création sur Notion d'un système de suivi des tickets (tracker)</t>
   </si>
   <si>
-    <t>Création dans Sitetracker d'un objet "évol et anomalies" pour la gestion des tickets</t>
-  </si>
-  <si>
     <t>Qualification des demandes (type, priorité), affectation, suivi, relance, clôture</t>
   </si>
   <si>
@@ -236,9 +215,6 @@
     <t>Dépannage réseau chez un particulier (box en surchauffe, redémarrage) – Granny &amp; Charly</t>
   </si>
   <si>
-    <t>Mise en place d'un serveur de messagerie – Granny &amp; Charly</t>
-  </si>
-  <si>
     <t>Diagnostic et résolution de problèmes de connexion, serveurs, comptes, sessions</t>
   </si>
   <si>
@@ -354,6 +330,30 @@
   </si>
   <si>
     <t>"08/2025 - 08/2026"</t>
+  </si>
+  <si>
+    <t>Recensement du parc informatique (matériel, VMs, logiciels, câblage) et Ticketing via GLPI</t>
+  </si>
+  <si>
+    <t>TP Suricata + Snort (IDS/IPS)</t>
+  </si>
+  <si>
+    <t>TP Zabbix + Nagios (supervision)</t>
+  </si>
+  <si>
+    <t>Création et gestion d'un outil de ticketing Salesforce</t>
+  </si>
+  <si>
+    <t>Conformité RGPD + Administration Sitetracker + Politique d'accès</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pilotage de la migration de données critiques Excel → Sitetracker. </t>
+  </si>
+  <si>
+    <t>Support technique et accompagnement des utilisateurs</t>
+  </si>
+  <si>
+    <t>Mise en place d'un serveur de messagerie et dépannage réseau  (Granny &amp; Charly)</t>
   </si>
 </sst>
 </file>
@@ -897,6 +897,9 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="17" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -962,9 +965,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="17" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1274,67 +1274,67 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AQ142"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.81640625" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:AQ144"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.85546875" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="70.453125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="26.7265625" style="1" customWidth="1"/>
-    <col min="3" max="8" width="18.7265625" style="1" customWidth="1"/>
-    <col min="9" max="43" width="11.453125" customWidth="1"/>
-    <col min="44" max="16384" width="10.81640625" style="1"/>
+    <col min="1" max="1" width="70.42578125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="26.7109375" style="1" customWidth="1"/>
+    <col min="3" max="8" width="18.7109375" style="1" customWidth="1"/>
+    <col min="9" max="43" width="11.42578125" customWidth="1"/>
+    <col min="44" max="16384" width="10.85546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:43" ht="40" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="24" t="s">
+    <row r="1" spans="1:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="25" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="24" t="s">
-        <v>96</v>
-      </c>
-      <c r="H1" s="24"/>
-    </row>
-    <row r="2" spans="1:43" ht="41.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="24" t="s">
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25" t="s">
+        <v>88</v>
+      </c>
+      <c r="H1" s="25"/>
+    </row>
+    <row r="2" spans="1:43" ht="41.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="25" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="24"/>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
-      <c r="F2" s="24"/>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24"/>
-    </row>
-    <row r="3" spans="1:43" ht="40" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="25" t="s">
+      <c r="B2" s="25"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
+      <c r="F2" s="25"/>
+      <c r="G2" s="25"/>
+      <c r="H2" s="25"/>
+    </row>
+    <row r="3" spans="1:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="26" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="26"/>
-      <c r="C3" s="26"/>
-      <c r="D3" s="26"/>
-      <c r="E3" s="27"/>
-      <c r="F3" s="31" t="s">
-        <v>97</v>
-      </c>
-      <c r="G3" s="26"/>
-      <c r="H3" s="32"/>
+      <c r="B3" s="27"/>
+      <c r="C3" s="27"/>
+      <c r="D3" s="27"/>
+      <c r="E3" s="28"/>
+      <c r="F3" s="32" t="s">
+        <v>89</v>
+      </c>
+      <c r="G3" s="27"/>
+      <c r="H3" s="33"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
-    <row r="4" spans="1:43" ht="40" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="28" t="s">
+    <row r="4" spans="1:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="29" t="s">
         <v>23</v>
       </c>
-      <c r="B4" s="29"/>
-      <c r="C4" s="29"/>
-      <c r="D4" s="29"/>
-      <c r="E4" s="30"/>
+      <c r="B4" s="30"/>
+      <c r="C4" s="30"/>
+      <c r="D4" s="30"/>
+      <c r="E4" s="31"/>
       <c r="F4" s="13" t="s">
         <v>8</v>
       </c>
@@ -1345,23 +1345,23 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:43" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="43" t="s">
-        <v>98</v>
-      </c>
-      <c r="B5" s="44"/>
-      <c r="C5" s="44"/>
-      <c r="D5" s="44"/>
-      <c r="E5" s="44"/>
-      <c r="F5" s="44"/>
-      <c r="G5" s="44"/>
-      <c r="H5" s="45"/>
-    </row>
-    <row r="6" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="33" t="s">
+    <row r="5" spans="1:43" ht="39.950000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="44" t="s">
+        <v>90</v>
+      </c>
+      <c r="B5" s="45"/>
+      <c r="C5" s="45"/>
+      <c r="D5" s="45"/>
+      <c r="E5" s="45"/>
+      <c r="F5" s="45"/>
+      <c r="G5" s="45"/>
+      <c r="H5" s="46"/>
+    </row>
+    <row r="6" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="34" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="41" t="s">
+      <c r="B6" s="42" t="s">
         <v>19</v>
       </c>
       <c r="C6" s="5" t="s">
@@ -1383,9 +1383,9 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:43" s="2" customFormat="1" ht="325" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="34"/>
-      <c r="B7" s="42"/>
+    <row r="7" spans="1:43" s="2" customFormat="1" ht="324.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="35"/>
+      <c r="B7" s="43"/>
       <c r="C7" s="7" t="s">
         <v>9</v>
       </c>
@@ -1440,17 +1440,17 @@
       <c r="AP7"/>
       <c r="AQ7"/>
     </row>
-    <row r="8" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.25">
-      <c r="A8" s="35" t="s">
+    <row r="8" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.2">
+      <c r="A8" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="B8" s="36"/>
-      <c r="C8" s="36"/>
-      <c r="D8" s="36"/>
-      <c r="E8" s="36"/>
-      <c r="F8" s="36"/>
-      <c r="G8" s="36"/>
-      <c r="H8" s="37"/>
+      <c r="B8" s="37"/>
+      <c r="C8" s="37"/>
+      <c r="D8" s="37"/>
+      <c r="E8" s="37"/>
+      <c r="F8" s="37"/>
+      <c r="G8" s="37"/>
+      <c r="H8" s="38"/>
       <c r="I8"/>
       <c r="J8"/>
       <c r="K8"/>
@@ -1487,18 +1487,18 @@
       <c r="AP8"/>
       <c r="AQ8"/>
     </row>
-    <row r="9" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="10" t="s">
-        <v>24</v>
+        <v>96</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>99</v>
+        <v>91</v>
       </c>
       <c r="C9" s="20"/>
       <c r="D9" s="14"/>
       <c r="E9" s="14"/>
       <c r="F9" s="14"/>
-      <c r="G9" s="14"/>
+      <c r="G9" s="22"/>
       <c r="H9" s="15"/>
       <c r="I9"/>
       <c r="J9"/>
@@ -1536,12 +1536,12 @@
       <c r="AP9"/>
       <c r="AQ9"/>
     </row>
-    <row r="10" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="10" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>99</v>
+        <v>91</v>
       </c>
       <c r="C10" s="20"/>
       <c r="D10" s="14"/>
@@ -1585,18 +1585,18 @@
       <c r="AP10"/>
       <c r="AQ10"/>
     </row>
-    <row r="11" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="10" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>99</v>
-      </c>
-      <c r="C11" s="20"/>
-      <c r="D11" s="14"/>
+        <v>93</v>
+      </c>
+      <c r="C11" s="22"/>
+      <c r="D11" s="22"/>
       <c r="E11" s="14"/>
       <c r="F11" s="14"/>
-      <c r="G11" s="14"/>
+      <c r="G11" s="22"/>
       <c r="H11" s="15"/>
       <c r="I11"/>
       <c r="J11"/>
@@ -1634,12 +1634,12 @@
       <c r="AP11"/>
       <c r="AQ11"/>
     </row>
-    <row r="12" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="10" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>99</v>
+        <v>91</v>
       </c>
       <c r="C12" s="20"/>
       <c r="D12" s="14"/>
@@ -1683,12 +1683,12 @@
       <c r="AP12"/>
       <c r="AQ12"/>
     </row>
-    <row r="13" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="10" t="s">
-        <v>47</v>
+        <v>33</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="C13" s="20"/>
       <c r="D13" s="14"/>
@@ -1732,12 +1732,12 @@
       <c r="AP13"/>
       <c r="AQ13"/>
     </row>
-    <row r="14" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="10" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="C14" s="20"/>
       <c r="D14" s="14"/>
@@ -1781,12 +1781,12 @@
       <c r="AP14"/>
       <c r="AQ14"/>
     </row>
-    <row r="15" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="10" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>99</v>
+        <v>91</v>
       </c>
       <c r="C15" s="20"/>
       <c r="D15" s="14"/>
@@ -1830,12 +1830,12 @@
       <c r="AP15"/>
       <c r="AQ15"/>
     </row>
-    <row r="16" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="10" t="s">
-        <v>50</v>
+        <v>97</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>99</v>
+        <v>91</v>
       </c>
       <c r="C16" s="20"/>
       <c r="D16" s="14"/>
@@ -1879,12 +1879,12 @@
       <c r="AP16"/>
       <c r="AQ16"/>
     </row>
-    <row r="17" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="10" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>99</v>
+        <v>91</v>
       </c>
       <c r="C17" s="20"/>
       <c r="D17" s="14"/>
@@ -1928,12 +1928,12 @@
       <c r="AP17"/>
       <c r="AQ17"/>
     </row>
-    <row r="18" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="10" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>99</v>
+        <v>91</v>
       </c>
       <c r="C18" s="20"/>
       <c r="D18" s="14"/>
@@ -1977,12 +1977,12 @@
       <c r="AP18"/>
       <c r="AQ18"/>
     </row>
-    <row r="19" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="10" t="s">
-        <v>53</v>
+        <v>98</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>99</v>
+        <v>91</v>
       </c>
       <c r="C19" s="20"/>
       <c r="D19" s="14"/>
@@ -2026,12 +2026,12 @@
       <c r="AP19"/>
       <c r="AQ19"/>
     </row>
-    <row r="20" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="10" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>101</v>
+        <v>91</v>
       </c>
       <c r="C20" s="20"/>
       <c r="D20" s="14"/>
@@ -2075,18 +2075,18 @@
       <c r="AP20"/>
       <c r="AQ20"/>
     </row>
-    <row r="21" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="10" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>101</v>
-      </c>
-      <c r="C21" s="14"/>
-      <c r="D21" s="22"/>
+        <v>93</v>
+      </c>
+      <c r="C21" s="20"/>
+      <c r="D21" s="14"/>
       <c r="E21" s="14"/>
       <c r="F21" s="14"/>
-      <c r="G21" s="22"/>
+      <c r="G21" s="14"/>
       <c r="H21" s="15"/>
       <c r="I21"/>
       <c r="J21"/>
@@ -2124,12 +2124,12 @@
       <c r="AP21"/>
       <c r="AQ21"/>
     </row>
-    <row r="22" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="10" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>101</v>
+        <v>93</v>
       </c>
       <c r="C22" s="14"/>
       <c r="D22" s="22"/>
@@ -2173,14 +2173,14 @@
       <c r="AP22"/>
       <c r="AQ22"/>
     </row>
-    <row r="23" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="10" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>101</v>
-      </c>
-      <c r="C23" s="14"/>
+        <v>93</v>
+      </c>
+      <c r="C23" s="22"/>
       <c r="D23" s="22"/>
       <c r="E23" s="14"/>
       <c r="F23" s="14"/>
@@ -2222,12 +2222,12 @@
       <c r="AP23"/>
       <c r="AQ23"/>
     </row>
-    <row r="24" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="10" t="s">
-        <v>62</v>
+        <v>54</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>101</v>
+        <v>93</v>
       </c>
       <c r="C24" s="14"/>
       <c r="D24" s="22"/>
@@ -2271,18 +2271,18 @@
       <c r="AP24"/>
       <c r="AQ24"/>
     </row>
-    <row r="25" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="10" t="s">
-        <v>69</v>
+        <v>55</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>101</v>
+        <v>93</v>
       </c>
       <c r="C25" s="14"/>
-      <c r="D25" s="14"/>
-      <c r="E25" s="22"/>
+      <c r="D25" s="22"/>
+      <c r="E25" s="14"/>
       <c r="F25" s="14"/>
-      <c r="G25" s="14"/>
+      <c r="G25" s="22"/>
       <c r="H25" s="15"/>
       <c r="I25"/>
       <c r="J25"/>
@@ -2320,12 +2320,12 @@
       <c r="AP25"/>
       <c r="AQ25"/>
     </row>
-    <row r="26" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="10" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>101</v>
+        <v>93</v>
       </c>
       <c r="C26" s="14"/>
       <c r="D26" s="14"/>
@@ -2369,18 +2369,18 @@
       <c r="AP26"/>
       <c r="AQ26"/>
     </row>
-    <row r="27" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="10" t="s">
-        <v>71</v>
+        <v>62</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>101</v>
+        <v>93</v>
       </c>
       <c r="C27" s="14"/>
       <c r="D27" s="14"/>
       <c r="E27" s="22"/>
       <c r="F27" s="14"/>
-      <c r="G27" s="14"/>
+      <c r="G27" s="22"/>
       <c r="H27" s="15"/>
       <c r="I27"/>
       <c r="J27"/>
@@ -2418,12 +2418,12 @@
       <c r="AP27"/>
       <c r="AQ27"/>
     </row>
-    <row r="28" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="10" t="s">
-        <v>72</v>
+        <v>63</v>
       </c>
       <c r="B28" s="9" t="s">
-        <v>101</v>
+        <v>93</v>
       </c>
       <c r="C28" s="14"/>
       <c r="D28" s="14"/>
@@ -2467,17 +2467,17 @@
       <c r="AP28"/>
       <c r="AQ28"/>
     </row>
-    <row r="29" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="10" t="s">
-        <v>73</v>
+        <v>64</v>
       </c>
       <c r="B29" s="9" t="s">
-        <v>101</v>
+        <v>93</v>
       </c>
       <c r="C29" s="14"/>
       <c r="D29" s="14"/>
       <c r="E29" s="22"/>
-      <c r="F29" s="14"/>
+      <c r="F29" s="22"/>
       <c r="G29" s="14"/>
       <c r="H29" s="15"/>
       <c r="I29"/>
@@ -2516,17 +2516,17 @@
       <c r="AP29"/>
       <c r="AQ29"/>
     </row>
-    <row r="30" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="10" t="s">
-        <v>74</v>
+        <v>65</v>
       </c>
       <c r="B30" s="9" t="s">
-        <v>101</v>
+        <v>93</v>
       </c>
       <c r="C30" s="14"/>
       <c r="D30" s="14"/>
       <c r="E30" s="22"/>
-      <c r="F30" s="14"/>
+      <c r="F30" s="22"/>
       <c r="G30" s="14"/>
       <c r="H30" s="15"/>
       <c r="I30"/>
@@ -2565,18 +2565,18 @@
       <c r="AP30"/>
       <c r="AQ30"/>
     </row>
-    <row r="31" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="10" t="s">
-        <v>75</v>
+        <v>66</v>
       </c>
       <c r="B31" s="9" t="s">
-        <v>101</v>
+        <v>93</v>
       </c>
       <c r="C31" s="14"/>
       <c r="D31" s="14"/>
       <c r="E31" s="22"/>
       <c r="F31" s="14"/>
-      <c r="G31" s="14"/>
+      <c r="G31" s="22"/>
       <c r="H31" s="15"/>
       <c r="I31"/>
       <c r="J31"/>
@@ -2614,18 +2614,18 @@
       <c r="AP31"/>
       <c r="AQ31"/>
     </row>
-    <row r="32" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="10" t="s">
-        <v>76</v>
+        <v>67</v>
       </c>
       <c r="B32" s="9" t="s">
-        <v>101</v>
+        <v>93</v>
       </c>
       <c r="C32" s="14"/>
       <c r="D32" s="14"/>
       <c r="E32" s="22"/>
-      <c r="F32" s="14"/>
-      <c r="G32" s="14"/>
+      <c r="F32" s="22"/>
+      <c r="G32" s="22"/>
       <c r="H32" s="15"/>
       <c r="I32"/>
       <c r="J32"/>
@@ -2663,19 +2663,19 @@
       <c r="AP32"/>
       <c r="AQ32"/>
     </row>
-    <row r="33" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="19" t="s">
-        <v>88</v>
+    <row r="33" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A33" s="10" t="s">
+        <v>68</v>
       </c>
       <c r="B33" s="9" t="s">
-        <v>101</v>
-      </c>
-      <c r="C33" s="12"/>
-      <c r="D33" s="12"/>
-      <c r="E33" s="12"/>
-      <c r="F33" s="21"/>
-      <c r="G33" s="12"/>
-      <c r="H33" s="16"/>
+        <v>93</v>
+      </c>
+      <c r="C33" s="14"/>
+      <c r="D33" s="14"/>
+      <c r="E33" s="22"/>
+      <c r="F33" s="14"/>
+      <c r="G33" s="22"/>
+      <c r="H33" s="15"/>
       <c r="I33"/>
       <c r="J33"/>
       <c r="K33"/>
@@ -2712,19 +2712,19 @@
       <c r="AP33"/>
       <c r="AQ33"/>
     </row>
-    <row r="34" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A34" s="19" t="s">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="B34" s="9" t="s">
-        <v>101</v>
+        <v>93</v>
       </c>
       <c r="C34" s="12"/>
       <c r="D34" s="12"/>
       <c r="E34" s="12"/>
-      <c r="F34" s="12"/>
+      <c r="F34" s="21"/>
       <c r="G34" s="12"/>
-      <c r="H34" s="23"/>
+      <c r="H34" s="16"/>
       <c r="I34"/>
       <c r="J34"/>
       <c r="K34"/>
@@ -2761,12 +2761,12 @@
       <c r="AP34"/>
       <c r="AQ34"/>
     </row>
-    <row r="35" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A35" s="19" t="s">
-        <v>89</v>
+        <v>82</v>
       </c>
       <c r="B35" s="9" t="s">
-        <v>101</v>
+        <v>93</v>
       </c>
       <c r="C35" s="12"/>
       <c r="D35" s="12"/>
@@ -2810,12 +2810,12 @@
       <c r="AP35"/>
       <c r="AQ35"/>
     </row>
-    <row r="36" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A36" s="19" t="s">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="B36" s="9" t="s">
-        <v>101</v>
+        <v>93</v>
       </c>
       <c r="C36" s="12"/>
       <c r="D36" s="12"/>
@@ -2859,12 +2859,12 @@
       <c r="AP36"/>
       <c r="AQ36"/>
     </row>
-    <row r="37" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A37" s="19" t="s">
-        <v>92</v>
+        <v>83</v>
       </c>
       <c r="B37" s="9" t="s">
-        <v>101</v>
+        <v>93</v>
       </c>
       <c r="C37" s="12"/>
       <c r="D37" s="12"/>
@@ -2908,12 +2908,12 @@
       <c r="AP37"/>
       <c r="AQ37"/>
     </row>
-    <row r="38" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A38" s="19" t="s">
+        <v>84</v>
+      </c>
+      <c r="B38" s="9" t="s">
         <v>93</v>
-      </c>
-      <c r="B38" s="9" t="s">
-        <v>101</v>
       </c>
       <c r="C38" s="12"/>
       <c r="D38" s="12"/>
@@ -2957,12 +2957,12 @@
       <c r="AP38"/>
       <c r="AQ38"/>
     </row>
-    <row r="39" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A39" s="19" t="s">
-        <v>94</v>
+        <v>85</v>
       </c>
       <c r="B39" s="9" t="s">
-        <v>101</v>
+        <v>93</v>
       </c>
       <c r="C39" s="12"/>
       <c r="D39" s="12"/>
@@ -3006,18 +3006,18 @@
       <c r="AP39"/>
       <c r="AQ39"/>
     </row>
-    <row r="40" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A40" s="19" t="s">
-        <v>95</v>
+        <v>86</v>
       </c>
       <c r="B40" s="9" t="s">
-        <v>101</v>
+        <v>93</v>
       </c>
       <c r="C40" s="12"/>
       <c r="D40" s="12"/>
       <c r="E40" s="12"/>
       <c r="F40" s="12"/>
-      <c r="G40" s="12"/>
+      <c r="G40" s="21"/>
       <c r="H40" s="23"/>
       <c r="I40"/>
       <c r="J40"/>
@@ -3055,15 +3055,19 @@
       <c r="AP40"/>
       <c r="AQ40"/>
     </row>
-    <row r="41" spans="1:43" s="2" customFormat="1" ht="40" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="10"/>
-      <c r="B41" s="9"/>
-      <c r="C41" s="14"/>
-      <c r="D41" s="14"/>
-      <c r="E41" s="14"/>
-      <c r="F41" s="14"/>
-      <c r="G41" s="14"/>
-      <c r="H41" s="15"/>
+    <row r="41" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="19" t="s">
+        <v>87</v>
+      </c>
+      <c r="B41" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="C41" s="21"/>
+      <c r="D41" s="12"/>
+      <c r="E41" s="12"/>
+      <c r="F41" s="12"/>
+      <c r="G41" s="21"/>
+      <c r="H41" s="23"/>
       <c r="I41"/>
       <c r="J41"/>
       <c r="K41"/>
@@ -3100,7 +3104,7 @@
       <c r="AP41"/>
       <c r="AQ41"/>
     </row>
-    <row r="42" spans="1:43" s="2" customFormat="1" ht="40" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="10"/>
       <c r="B42" s="9"/>
       <c r="C42" s="14"/>
@@ -3145,17 +3149,15 @@
       <c r="AP42"/>
       <c r="AQ42"/>
     </row>
-    <row r="43" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.25">
-      <c r="A43" s="38" t="s">
-        <v>20</v>
-      </c>
-      <c r="B43" s="39"/>
-      <c r="C43" s="39"/>
-      <c r="D43" s="39"/>
-      <c r="E43" s="39"/>
-      <c r="F43" s="39"/>
-      <c r="G43" s="39"/>
-      <c r="H43" s="40"/>
+    <row r="43" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A43" s="10"/>
+      <c r="B43" s="9"/>
+      <c r="C43" s="14"/>
+      <c r="D43" s="14"/>
+      <c r="E43" s="14"/>
+      <c r="F43" s="14"/>
+      <c r="G43" s="14"/>
+      <c r="H43" s="15"/>
       <c r="I43"/>
       <c r="J43"/>
       <c r="K43"/>
@@ -3192,19 +3194,17 @@
       <c r="AP43"/>
       <c r="AQ43"/>
     </row>
-    <row r="44" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="B44" s="9" t="s">
-        <v>102</v>
-      </c>
-      <c r="C44" s="20"/>
-      <c r="D44" s="14"/>
-      <c r="E44" s="14"/>
-      <c r="F44" s="14"/>
-      <c r="G44" s="14"/>
-      <c r="H44" s="15"/>
+    <row r="44" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.2">
+      <c r="A44" s="39" t="s">
+        <v>20</v>
+      </c>
+      <c r="B44" s="40"/>
+      <c r="C44" s="40"/>
+      <c r="D44" s="40"/>
+      <c r="E44" s="40"/>
+      <c r="F44" s="40"/>
+      <c r="G44" s="40"/>
+      <c r="H44" s="41"/>
       <c r="I44"/>
       <c r="J44"/>
       <c r="K44"/>
@@ -3241,12 +3241,12 @@
       <c r="AP44"/>
       <c r="AQ44"/>
     </row>
-    <row r="45" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="10" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B45" s="9" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
       <c r="C45" s="20"/>
       <c r="D45" s="14"/>
@@ -3290,12 +3290,12 @@
       <c r="AP45"/>
       <c r="AQ45"/>
     </row>
-    <row r="46" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="10" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B46" s="9" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
       <c r="C46" s="20"/>
       <c r="D46" s="14"/>
@@ -3339,12 +3339,12 @@
       <c r="AP46"/>
       <c r="AQ46"/>
     </row>
-    <row r="47" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="10" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B47" s="9" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
       <c r="C47" s="20"/>
       <c r="D47" s="14"/>
@@ -3388,12 +3388,12 @@
       <c r="AP47"/>
       <c r="AQ47"/>
     </row>
-    <row r="48" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="10" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B48" s="9" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
       <c r="C48" s="20"/>
       <c r="D48" s="14"/>
@@ -3437,12 +3437,12 @@
       <c r="AP48"/>
       <c r="AQ48"/>
     </row>
-    <row r="49" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="10" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="B49" s="9" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
       <c r="C49" s="20"/>
       <c r="D49" s="14"/>
@@ -3486,12 +3486,12 @@
       <c r="AP49"/>
       <c r="AQ49"/>
     </row>
-    <row r="50" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="10" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="B50" s="9" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
       <c r="C50" s="20"/>
       <c r="D50" s="14"/>
@@ -3535,12 +3535,12 @@
       <c r="AP50"/>
       <c r="AQ50"/>
     </row>
-    <row r="51" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="10" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B51" s="9" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
       <c r="C51" s="20"/>
       <c r="D51" s="14"/>
@@ -3584,18 +3584,18 @@
       <c r="AP51"/>
       <c r="AQ51"/>
     </row>
-    <row r="52" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="10" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="B52" s="9" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
       <c r="C52" s="20"/>
       <c r="D52" s="14"/>
       <c r="E52" s="14"/>
       <c r="F52" s="14"/>
-      <c r="G52" s="14"/>
+      <c r="G52" s="22"/>
       <c r="H52" s="15"/>
       <c r="I52"/>
       <c r="J52"/>
@@ -3633,12 +3633,12 @@
       <c r="AP52"/>
       <c r="AQ52"/>
     </row>
-    <row r="53" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="10" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="B53" s="9" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
       <c r="C53" s="20"/>
       <c r="D53" s="14"/>
@@ -3682,12 +3682,12 @@
       <c r="AP53"/>
       <c r="AQ53"/>
     </row>
-    <row r="54" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="10" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="B54" s="9" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
       <c r="C54" s="20"/>
       <c r="D54" s="14"/>
@@ -3731,18 +3731,18 @@
       <c r="AP54"/>
       <c r="AQ54"/>
     </row>
-    <row r="55" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="10" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="B55" s="9" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
       <c r="C55" s="20"/>
       <c r="D55" s="14"/>
       <c r="E55" s="14"/>
       <c r="F55" s="14"/>
-      <c r="G55" s="14"/>
+      <c r="G55" s="22"/>
       <c r="H55" s="15"/>
       <c r="I55"/>
       <c r="J55"/>
@@ -3780,10 +3780,14 @@
       <c r="AP55"/>
       <c r="AQ55"/>
     </row>
-    <row r="56" spans="1:43" s="2" customFormat="1" ht="40" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="10"/>
-      <c r="B56" s="9"/>
-      <c r="C56" s="14"/>
+    <row r="56" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A56" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="B56" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="C56" s="20"/>
       <c r="D56" s="14"/>
       <c r="E56" s="14"/>
       <c r="F56" s="14"/>
@@ -3825,7 +3829,7 @@
       <c r="AP56"/>
       <c r="AQ56"/>
     </row>
-    <row r="57" spans="1:43" s="2" customFormat="1" ht="40" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="10"/>
       <c r="B57" s="9"/>
       <c r="C57" s="14"/>
@@ -3870,17 +3874,15 @@
       <c r="AP57"/>
       <c r="AQ57"/>
     </row>
-    <row r="58" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.25">
-      <c r="A58" s="38" t="s">
-        <v>21</v>
-      </c>
-      <c r="B58" s="39"/>
-      <c r="C58" s="39"/>
-      <c r="D58" s="39"/>
-      <c r="E58" s="39"/>
-      <c r="F58" s="39"/>
-      <c r="G58" s="39"/>
-      <c r="H58" s="40"/>
+    <row r="58" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A58" s="10"/>
+      <c r="B58" s="9"/>
+      <c r="C58" s="14"/>
+      <c r="D58" s="14"/>
+      <c r="E58" s="14"/>
+      <c r="F58" s="14"/>
+      <c r="G58" s="14"/>
+      <c r="H58" s="15"/>
       <c r="I58"/>
       <c r="J58"/>
       <c r="K58"/>
@@ -3917,19 +3919,17 @@
       <c r="AP58"/>
       <c r="AQ58"/>
     </row>
-    <row r="59" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="B59" s="46" t="s">
-        <v>103</v>
-      </c>
-      <c r="C59" s="20"/>
-      <c r="D59" s="14"/>
-      <c r="E59" s="14"/>
-      <c r="F59" s="14"/>
-      <c r="G59" s="14"/>
-      <c r="H59" s="15"/>
+    <row r="59" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.2">
+      <c r="A59" s="39" t="s">
+        <v>21</v>
+      </c>
+      <c r="B59" s="40"/>
+      <c r="C59" s="40"/>
+      <c r="D59" s="40"/>
+      <c r="E59" s="40"/>
+      <c r="F59" s="40"/>
+      <c r="G59" s="40"/>
+      <c r="H59" s="41"/>
       <c r="I59"/>
       <c r="J59"/>
       <c r="K59"/>
@@ -3966,15 +3966,15 @@
       <c r="AP59"/>
       <c r="AQ59"/>
     </row>
-    <row r="60" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="10" t="s">
-        <v>34</v>
-      </c>
-      <c r="B60" s="46" t="s">
-        <v>103</v>
+        <v>100</v>
+      </c>
+      <c r="B60" s="24" t="s">
+        <v>95</v>
       </c>
       <c r="C60" s="20"/>
-      <c r="D60" s="14"/>
+      <c r="D60" s="22"/>
       <c r="E60" s="14"/>
       <c r="F60" s="14"/>
       <c r="G60" s="14"/>
@@ -4015,18 +4015,18 @@
       <c r="AP60"/>
       <c r="AQ60"/>
     </row>
-    <row r="61" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="10" t="s">
-        <v>35</v>
-      </c>
-      <c r="B61" s="46" t="s">
-        <v>103</v>
+        <v>101</v>
+      </c>
+      <c r="B61" s="24" t="s">
+        <v>95</v>
       </c>
       <c r="C61" s="20"/>
       <c r="D61" s="14"/>
       <c r="E61" s="14"/>
       <c r="F61" s="14"/>
-      <c r="G61" s="14"/>
+      <c r="G61" s="22"/>
       <c r="H61" s="15"/>
       <c r="I61"/>
       <c r="J61"/>
@@ -4064,12 +4064,12 @@
       <c r="AP61"/>
       <c r="AQ61"/>
     </row>
-    <row r="62" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="10" t="s">
-        <v>41</v>
-      </c>
-      <c r="B62" s="46" t="s">
-        <v>103</v>
+        <v>32</v>
+      </c>
+      <c r="B62" s="24" t="s">
+        <v>95</v>
       </c>
       <c r="C62" s="20"/>
       <c r="D62" s="14"/>
@@ -4113,12 +4113,12 @@
       <c r="AP62"/>
       <c r="AQ62"/>
     </row>
-    <row r="63" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="10" t="s">
-        <v>40</v>
-      </c>
-      <c r="B63" s="46" t="s">
-        <v>103</v>
+        <v>38</v>
+      </c>
+      <c r="B63" s="24" t="s">
+        <v>95</v>
       </c>
       <c r="C63" s="20"/>
       <c r="D63" s="14"/>
@@ -4162,18 +4162,18 @@
       <c r="AP63"/>
       <c r="AQ63"/>
     </row>
-    <row r="64" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="10" t="s">
-        <v>42</v>
-      </c>
-      <c r="B64" s="46" t="s">
-        <v>103</v>
+        <v>37</v>
+      </c>
+      <c r="B64" s="24" t="s">
+        <v>95</v>
       </c>
       <c r="C64" s="20"/>
       <c r="D64" s="14"/>
       <c r="E64" s="14"/>
       <c r="F64" s="14"/>
-      <c r="G64" s="14"/>
+      <c r="G64" s="22"/>
       <c r="H64" s="15"/>
       <c r="I64"/>
       <c r="J64"/>
@@ -4211,19 +4211,19 @@
       <c r="AP64"/>
       <c r="AQ64"/>
     </row>
-    <row r="65" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A65" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="B65" s="46" t="s">
-        <v>103</v>
+    <row r="65" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A65" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="B65" s="24" t="s">
+        <v>95</v>
       </c>
       <c r="C65" s="20"/>
-      <c r="D65" s="12"/>
-      <c r="E65" s="12"/>
-      <c r="F65" s="12"/>
-      <c r="G65" s="12"/>
-      <c r="H65" s="16"/>
+      <c r="D65" s="14"/>
+      <c r="E65" s="14"/>
+      <c r="F65" s="14"/>
+      <c r="G65" s="14"/>
+      <c r="H65" s="15"/>
       <c r="I65"/>
       <c r="J65"/>
       <c r="K65"/>
@@ -4260,15 +4260,15 @@
       <c r="AP65"/>
       <c r="AQ65"/>
     </row>
-    <row r="66" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A66" s="19" t="s">
-        <v>57</v>
-      </c>
-      <c r="B66" s="46" t="s">
-        <v>103</v>
-      </c>
-      <c r="C66" s="12"/>
-      <c r="D66" s="21"/>
+    <row r="66" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A66" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="B66" s="24" t="s">
+        <v>95</v>
+      </c>
+      <c r="C66" s="20"/>
+      <c r="D66" s="12"/>
       <c r="E66" s="12"/>
       <c r="F66" s="12"/>
       <c r="G66" s="12"/>
@@ -4309,17 +4309,17 @@
       <c r="AP66"/>
       <c r="AQ66"/>
     </row>
-    <row r="67" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A67" s="19" t="s">
-        <v>58</v>
-      </c>
-      <c r="B67" s="46" t="s">
-        <v>103</v>
+        <v>99</v>
+      </c>
+      <c r="B67" s="24" t="s">
+        <v>95</v>
       </c>
       <c r="C67" s="12"/>
       <c r="D67" s="21"/>
       <c r="E67" s="12"/>
-      <c r="F67" s="12"/>
+      <c r="F67" s="21"/>
       <c r="G67" s="12"/>
       <c r="H67" s="16"/>
       <c r="I67"/>
@@ -4358,12 +4358,12 @@
       <c r="AP67"/>
       <c r="AQ67"/>
     </row>
-    <row r="68" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A68" s="19" t="s">
-        <v>59</v>
-      </c>
-      <c r="B68" s="46" t="s">
-        <v>103</v>
+        <v>52</v>
+      </c>
+      <c r="B68" s="24" t="s">
+        <v>95</v>
       </c>
       <c r="C68" s="12"/>
       <c r="D68" s="21"/>
@@ -4407,12 +4407,12 @@
       <c r="AP68"/>
       <c r="AQ68"/>
     </row>
-    <row r="69" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A69" s="19" t="s">
-        <v>60</v>
-      </c>
-      <c r="B69" s="46" t="s">
-        <v>103</v>
+        <v>102</v>
+      </c>
+      <c r="B69" s="24" t="s">
+        <v>95</v>
       </c>
       <c r="C69" s="12"/>
       <c r="D69" s="21"/>
@@ -4456,12 +4456,12 @@
       <c r="AP69"/>
       <c r="AQ69"/>
     </row>
-    <row r="70" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A70" s="19" t="s">
-        <v>63</v>
-      </c>
-      <c r="B70" s="46" t="s">
-        <v>103</v>
+        <v>53</v>
+      </c>
+      <c r="B70" s="24" t="s">
+        <v>95</v>
       </c>
       <c r="C70" s="12"/>
       <c r="D70" s="21"/>
@@ -4505,12 +4505,12 @@
       <c r="AP70"/>
       <c r="AQ70"/>
     </row>
-    <row r="71" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A71" s="19" t="s">
-        <v>64</v>
-      </c>
-      <c r="B71" s="46" t="s">
-        <v>103</v>
+        <v>56</v>
+      </c>
+      <c r="B71" s="24" t="s">
+        <v>95</v>
       </c>
       <c r="C71" s="12"/>
       <c r="D71" s="21"/>
@@ -4554,18 +4554,18 @@
       <c r="AP71"/>
       <c r="AQ71"/>
     </row>
-    <row r="72" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A72" s="19" t="s">
-        <v>65</v>
-      </c>
-      <c r="B72" s="46" t="s">
-        <v>103</v>
-      </c>
-      <c r="C72" s="12"/>
+        <v>59</v>
+      </c>
+      <c r="B72" s="24" t="s">
+        <v>95</v>
+      </c>
+      <c r="C72" s="21"/>
       <c r="D72" s="21"/>
       <c r="E72" s="12"/>
       <c r="F72" s="12"/>
-      <c r="G72" s="12"/>
+      <c r="G72" s="21"/>
       <c r="H72" s="16"/>
       <c r="I72"/>
       <c r="J72"/>
@@ -4603,18 +4603,18 @@
       <c r="AP72"/>
       <c r="AQ72"/>
     </row>
-    <row r="73" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A73" s="19" t="s">
-        <v>66</v>
-      </c>
-      <c r="B73" s="46" t="s">
         <v>103</v>
       </c>
-      <c r="C73" s="12"/>
+      <c r="B73" s="24" t="s">
+        <v>95</v>
+      </c>
+      <c r="C73" s="21"/>
       <c r="D73" s="21"/>
       <c r="E73" s="12"/>
       <c r="F73" s="12"/>
-      <c r="G73" s="12"/>
+      <c r="G73" s="21"/>
       <c r="H73" s="16"/>
       <c r="I73"/>
       <c r="J73"/>
@@ -4652,14 +4652,14 @@
       <c r="AP73"/>
       <c r="AQ73"/>
     </row>
-    <row r="74" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A74" s="19" t="s">
-        <v>67</v>
-      </c>
-      <c r="B74" s="46" t="s">
-        <v>103</v>
-      </c>
-      <c r="C74" s="12"/>
+        <v>57</v>
+      </c>
+      <c r="B74" s="24" t="s">
+        <v>95</v>
+      </c>
+      <c r="C74" s="21"/>
       <c r="D74" s="21"/>
       <c r="E74" s="12"/>
       <c r="F74" s="12"/>
@@ -4701,14 +4701,14 @@
       <c r="AP74"/>
       <c r="AQ74"/>
     </row>
-    <row r="75" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A75" s="19" t="s">
-        <v>68</v>
-      </c>
-      <c r="B75" s="46" t="s">
-        <v>103</v>
-      </c>
-      <c r="C75" s="12"/>
+        <v>58</v>
+      </c>
+      <c r="B75" s="24" t="s">
+        <v>95</v>
+      </c>
+      <c r="C75" s="21"/>
       <c r="D75" s="21"/>
       <c r="E75" s="12"/>
       <c r="F75" s="12"/>
@@ -4750,16 +4750,16 @@
       <c r="AP75"/>
       <c r="AQ75"/>
     </row>
-    <row r="76" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A76" s="19" t="s">
-        <v>77</v>
-      </c>
-      <c r="B76" s="46" t="s">
-        <v>103</v>
-      </c>
-      <c r="C76" s="12"/>
-      <c r="D76" s="12"/>
-      <c r="E76" s="21"/>
+        <v>59</v>
+      </c>
+      <c r="B76" s="24" t="s">
+        <v>95</v>
+      </c>
+      <c r="C76" s="21"/>
+      <c r="D76" s="21"/>
+      <c r="E76" s="12"/>
       <c r="F76" s="12"/>
       <c r="G76" s="12"/>
       <c r="H76" s="16"/>
@@ -4799,17 +4799,17 @@
       <c r="AP76"/>
       <c r="AQ76"/>
     </row>
-    <row r="77" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A77" s="19" t="s">
-        <v>78</v>
-      </c>
-      <c r="B77" s="46" t="s">
-        <v>103</v>
+        <v>60</v>
+      </c>
+      <c r="B77" s="24" t="s">
+        <v>95</v>
       </c>
       <c r="C77" s="12"/>
-      <c r="D77" s="12"/>
-      <c r="E77" s="21"/>
-      <c r="F77" s="12"/>
+      <c r="D77" s="21"/>
+      <c r="E77" s="12"/>
+      <c r="F77" s="21"/>
       <c r="G77" s="12"/>
       <c r="H77" s="16"/>
       <c r="I77"/>
@@ -4848,17 +4848,17 @@
       <c r="AP77"/>
       <c r="AQ77"/>
     </row>
-    <row r="78" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A78" s="19" t="s">
-        <v>79</v>
-      </c>
-      <c r="B78" s="46" t="s">
-        <v>103</v>
+        <v>69</v>
+      </c>
+      <c r="B78" s="24" t="s">
+        <v>95</v>
       </c>
       <c r="C78" s="12"/>
       <c r="D78" s="12"/>
-      <c r="E78" s="21"/>
-      <c r="F78" s="12"/>
+      <c r="E78" s="12"/>
+      <c r="F78" s="21"/>
       <c r="G78" s="12"/>
       <c r="H78" s="16"/>
       <c r="I78"/>
@@ -4897,17 +4897,17 @@
       <c r="AP78"/>
       <c r="AQ78"/>
     </row>
-    <row r="79" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A79" s="19" t="s">
-        <v>80</v>
-      </c>
-      <c r="B79" s="46" t="s">
-        <v>103</v>
+        <v>70</v>
+      </c>
+      <c r="B79" s="24" t="s">
+        <v>95</v>
       </c>
       <c r="C79" s="12"/>
       <c r="D79" s="12"/>
-      <c r="E79" s="21"/>
-      <c r="F79" s="12"/>
+      <c r="E79" s="12"/>
+      <c r="F79" s="21"/>
       <c r="G79" s="12"/>
       <c r="H79" s="16"/>
       <c r="I79"/>
@@ -4946,17 +4946,17 @@
       <c r="AP79"/>
       <c r="AQ79"/>
     </row>
-    <row r="80" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A80" s="19" t="s">
-        <v>81</v>
-      </c>
-      <c r="B80" s="46" t="s">
-        <v>103</v>
+        <v>71</v>
+      </c>
+      <c r="B80" s="24" t="s">
+        <v>95</v>
       </c>
       <c r="C80" s="12"/>
       <c r="D80" s="12"/>
-      <c r="E80" s="21"/>
-      <c r="F80" s="12"/>
+      <c r="E80" s="12"/>
+      <c r="F80" s="21"/>
       <c r="G80" s="12"/>
       <c r="H80" s="16"/>
       <c r="I80"/>
@@ -4995,17 +4995,17 @@
       <c r="AP80"/>
       <c r="AQ80"/>
     </row>
-    <row r="81" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A81" s="19" t="s">
-        <v>82</v>
-      </c>
-      <c r="B81" s="46" t="s">
-        <v>103</v>
+        <v>72</v>
+      </c>
+      <c r="B81" s="24" t="s">
+        <v>95</v>
       </c>
       <c r="C81" s="12"/>
       <c r="D81" s="12"/>
-      <c r="E81" s="21"/>
-      <c r="F81" s="12"/>
+      <c r="E81" s="12"/>
+      <c r="F81" s="21"/>
       <c r="G81" s="12"/>
       <c r="H81" s="16"/>
       <c r="I81"/>
@@ -5044,12 +5044,12 @@
       <c r="AP81"/>
       <c r="AQ81"/>
     </row>
-    <row r="82" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A82" s="19" t="s">
-        <v>83</v>
-      </c>
-      <c r="B82" s="46" t="s">
-        <v>103</v>
+        <v>73</v>
+      </c>
+      <c r="B82" s="24" t="s">
+        <v>95</v>
       </c>
       <c r="C82" s="12"/>
       <c r="D82" s="12"/>
@@ -5093,12 +5093,12 @@
       <c r="AP82"/>
       <c r="AQ82"/>
     </row>
-    <row r="83" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A83" s="19" t="s">
-        <v>84</v>
-      </c>
-      <c r="B83" s="46" t="s">
-        <v>103</v>
+        <v>74</v>
+      </c>
+      <c r="B83" s="24" t="s">
+        <v>95</v>
       </c>
       <c r="C83" s="12"/>
       <c r="D83" s="12"/>
@@ -5142,18 +5142,18 @@
       <c r="AP83"/>
       <c r="AQ83"/>
     </row>
-    <row r="84" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A84" s="19" t="s">
-        <v>85</v>
-      </c>
-      <c r="B84" s="46" t="s">
-        <v>103</v>
+        <v>75</v>
+      </c>
+      <c r="B84" s="24" t="s">
+        <v>95</v>
       </c>
       <c r="C84" s="12"/>
       <c r="D84" s="12"/>
       <c r="E84" s="12"/>
-      <c r="F84" s="21"/>
-      <c r="G84" s="12"/>
+      <c r="F84" s="12"/>
+      <c r="G84" s="21"/>
       <c r="H84" s="16"/>
       <c r="I84"/>
       <c r="J84"/>
@@ -5191,18 +5191,18 @@
       <c r="AP84"/>
       <c r="AQ84"/>
     </row>
-    <row r="85" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A85" s="19" t="s">
-        <v>87</v>
-      </c>
-      <c r="B85" s="46" t="s">
-        <v>103</v>
+        <v>76</v>
+      </c>
+      <c r="B85" s="24" t="s">
+        <v>95</v>
       </c>
       <c r="C85" s="12"/>
       <c r="D85" s="12"/>
       <c r="E85" s="12"/>
-      <c r="F85" s="21"/>
-      <c r="G85" s="12"/>
+      <c r="F85" s="12"/>
+      <c r="G85" s="21"/>
       <c r="H85" s="16"/>
       <c r="I85"/>
       <c r="J85"/>
@@ -5240,14 +5240,14 @@
       <c r="AP85"/>
       <c r="AQ85"/>
     </row>
-    <row r="86" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A86" s="19" t="s">
-        <v>86</v>
-      </c>
-      <c r="B86" s="46" t="s">
-        <v>103</v>
-      </c>
-      <c r="C86" s="12"/>
+        <v>77</v>
+      </c>
+      <c r="B86" s="24" t="s">
+        <v>95</v>
+      </c>
+      <c r="C86" s="21"/>
       <c r="D86" s="12"/>
       <c r="E86" s="12"/>
       <c r="F86" s="12"/>
@@ -5289,14 +5289,18 @@
       <c r="AP86"/>
       <c r="AQ86"/>
     </row>
-    <row r="87" spans="1:43" s="2" customFormat="1" ht="40" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A87" s="19"/>
-      <c r="B87" s="12"/>
+    <row r="87" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A87" s="19" t="s">
+        <v>79</v>
+      </c>
+      <c r="B87" s="24" t="s">
+        <v>95</v>
+      </c>
       <c r="C87" s="12"/>
-      <c r="D87" s="12"/>
+      <c r="D87" s="21"/>
       <c r="E87" s="12"/>
       <c r="F87" s="12"/>
-      <c r="G87" s="12"/>
+      <c r="G87" s="21"/>
       <c r="H87" s="16"/>
       <c r="I87"/>
       <c r="J87"/>
@@ -5334,14 +5338,18 @@
       <c r="AP87"/>
       <c r="AQ87"/>
     </row>
-    <row r="88" spans="1:43" s="2" customFormat="1" ht="40" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A88" s="19"/>
-      <c r="B88" s="12"/>
+    <row r="88" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A88" s="19" t="s">
+        <v>78</v>
+      </c>
+      <c r="B88" s="24" t="s">
+        <v>95</v>
+      </c>
       <c r="C88" s="12"/>
-      <c r="D88" s="12"/>
+      <c r="D88" s="21"/>
       <c r="E88" s="12"/>
       <c r="F88" s="12"/>
-      <c r="G88" s="12"/>
+      <c r="G88" s="21"/>
       <c r="H88" s="16"/>
       <c r="I88"/>
       <c r="J88"/>
@@ -5379,9 +5387,9 @@
       <c r="AP88"/>
       <c r="AQ88"/>
     </row>
-    <row r="89" spans="1:43" s="2" customFormat="1" ht="40" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A89" s="19" t="s">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="B89" s="12"/>
       <c r="C89" s="12"/>
@@ -5426,9 +5434,9 @@
       <c r="AP89"/>
       <c r="AQ89"/>
     </row>
-    <row r="90" spans="1:43" s="2" customFormat="1" ht="40" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A90" s="19" t="s">
-        <v>91</v>
+        <v>78</v>
       </c>
       <c r="B90" s="12"/>
       <c r="C90" s="12"/>
@@ -5473,9 +5481,9 @@
       <c r="AP90"/>
       <c r="AQ90"/>
     </row>
-    <row r="91" spans="1:43" s="2" customFormat="1" ht="40" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A91" s="19" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
       <c r="B91" s="12"/>
       <c r="C91" s="12"/>
@@ -5520,9 +5528,9 @@
       <c r="AP91"/>
       <c r="AQ91"/>
     </row>
-    <row r="92" spans="1:43" s="2" customFormat="1" ht="40" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A92" s="19" t="s">
-        <v>93</v>
+        <v>78</v>
       </c>
       <c r="B92" s="12"/>
       <c r="C92" s="12"/>
@@ -5567,9 +5575,9 @@
       <c r="AP92"/>
       <c r="AQ92"/>
     </row>
-    <row r="93" spans="1:43" s="2" customFormat="1" ht="40" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A93" s="19" t="s">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="B93" s="12"/>
       <c r="C93" s="12"/>
@@ -5614,9 +5622,9 @@
       <c r="AP93"/>
       <c r="AQ93"/>
     </row>
-    <row r="94" spans="1:43" s="2" customFormat="1" ht="40" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A94" s="19" t="s">
-        <v>95</v>
+        <v>78</v>
       </c>
       <c r="B94" s="12"/>
       <c r="C94" s="12"/>
@@ -5661,15 +5669,17 @@
       <c r="AP94"/>
       <c r="AQ94"/>
     </row>
-    <row r="95" spans="1:43" s="2" customFormat="1" ht="14" x14ac:dyDescent="0.25">
-      <c r="A95" s="19"/>
-      <c r="B95" s="3"/>
-      <c r="C95" s="4"/>
-      <c r="D95" s="4"/>
-      <c r="E95" s="4"/>
-      <c r="F95" s="4"/>
-      <c r="G95" s="4"/>
-      <c r="H95" s="4"/>
+    <row r="95" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A95" s="19" t="s">
+        <v>78</v>
+      </c>
+      <c r="B95" s="12"/>
+      <c r="C95" s="12"/>
+      <c r="D95" s="12"/>
+      <c r="E95" s="12"/>
+      <c r="F95" s="12"/>
+      <c r="G95" s="12"/>
+      <c r="H95" s="16"/>
       <c r="I95"/>
       <c r="J95"/>
       <c r="K95"/>
@@ -5706,15 +5716,17 @@
       <c r="AP95"/>
       <c r="AQ95"/>
     </row>
-    <row r="96" spans="1:43" s="2" customFormat="1" ht="14" x14ac:dyDescent="0.25">
-      <c r="A96" s="19"/>
-      <c r="B96" s="3"/>
-      <c r="C96" s="4"/>
-      <c r="D96" s="4"/>
-      <c r="E96" s="4"/>
-      <c r="F96" s="4"/>
-      <c r="G96" s="4"/>
-      <c r="H96" s="4"/>
+    <row r="96" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A96" s="19" t="s">
+        <v>78</v>
+      </c>
+      <c r="B96" s="12"/>
+      <c r="C96" s="12"/>
+      <c r="D96" s="12"/>
+      <c r="E96" s="12"/>
+      <c r="F96" s="12"/>
+      <c r="G96" s="12"/>
+      <c r="H96" s="16"/>
       <c r="I96"/>
       <c r="J96"/>
       <c r="K96"/>
@@ -5751,71 +5763,161 @@
       <c r="AP96"/>
       <c r="AQ96"/>
     </row>
-    <row r="97" spans="1:1" customFormat="1" ht="14" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:43" s="2" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A97" s="19"/>
-    </row>
-    <row r="98" spans="1:1" customFormat="1" ht="14" x14ac:dyDescent="0.25">
+      <c r="B97" s="3"/>
+      <c r="C97" s="4"/>
+      <c r="D97" s="4"/>
+      <c r="E97" s="4"/>
+      <c r="F97" s="4"/>
+      <c r="G97" s="4"/>
+      <c r="H97" s="4"/>
+      <c r="I97"/>
+      <c r="J97"/>
+      <c r="K97"/>
+      <c r="L97"/>
+      <c r="M97"/>
+      <c r="N97"/>
+      <c r="O97"/>
+      <c r="P97"/>
+      <c r="Q97"/>
+      <c r="R97"/>
+      <c r="S97"/>
+      <c r="T97"/>
+      <c r="U97"/>
+      <c r="V97"/>
+      <c r="W97"/>
+      <c r="X97"/>
+      <c r="Y97"/>
+      <c r="Z97"/>
+      <c r="AA97"/>
+      <c r="AB97"/>
+      <c r="AC97"/>
+      <c r="AD97"/>
+      <c r="AE97"/>
+      <c r="AF97"/>
+      <c r="AG97"/>
+      <c r="AH97"/>
+      <c r="AI97"/>
+      <c r="AJ97"/>
+      <c r="AK97"/>
+      <c r="AL97"/>
+      <c r="AM97"/>
+      <c r="AN97"/>
+      <c r="AO97"/>
+      <c r="AP97"/>
+      <c r="AQ97"/>
+    </row>
+    <row r="98" spans="1:43" s="2" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A98" s="19"/>
-    </row>
-    <row r="99" spans="1:1" customFormat="1" ht="14" x14ac:dyDescent="0.25">
+      <c r="B98" s="3"/>
+      <c r="C98" s="4"/>
+      <c r="D98" s="4"/>
+      <c r="E98" s="4"/>
+      <c r="F98" s="4"/>
+      <c r="G98" s="4"/>
+      <c r="H98" s="4"/>
+      <c r="I98"/>
+      <c r="J98"/>
+      <c r="K98"/>
+      <c r="L98"/>
+      <c r="M98"/>
+      <c r="N98"/>
+      <c r="O98"/>
+      <c r="P98"/>
+      <c r="Q98"/>
+      <c r="R98"/>
+      <c r="S98"/>
+      <c r="T98"/>
+      <c r="U98"/>
+      <c r="V98"/>
+      <c r="W98"/>
+      <c r="X98"/>
+      <c r="Y98"/>
+      <c r="Z98"/>
+      <c r="AA98"/>
+      <c r="AB98"/>
+      <c r="AC98"/>
+      <c r="AD98"/>
+      <c r="AE98"/>
+      <c r="AF98"/>
+      <c r="AG98"/>
+      <c r="AH98"/>
+      <c r="AI98"/>
+      <c r="AJ98"/>
+      <c r="AK98"/>
+      <c r="AL98"/>
+      <c r="AM98"/>
+      <c r="AN98"/>
+      <c r="AO98"/>
+      <c r="AP98"/>
+      <c r="AQ98"/>
+    </row>
+    <row r="99" spans="1:43" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A99" s="19"/>
     </row>
-    <row r="100" spans="1:1" customFormat="1" ht="14" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:43" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A100" s="19"/>
     </row>
-    <row r="101" spans="1:1" customFormat="1" ht="14" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:43" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A101" s="19"/>
     </row>
-    <row r="102" spans="1:1" customFormat="1" ht="14" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:43" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A102" s="19"/>
     </row>
-    <row r="103" spans="1:1" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="104" spans="1:1" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="105" spans="1:1" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="106" spans="1:1" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="107" spans="1:1" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="108" spans="1:1" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="109" spans="1:1" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="110" spans="1:1" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="111" spans="1:1" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="112" spans="1:1" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="113" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="114" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="115" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="116" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="117" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="118" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="119" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="120" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="121" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="122" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="123" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="124" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="125" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="126" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="127" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="128" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="129" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="130" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="131" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="132" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="133" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="134" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="135" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="136" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="137" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="138" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="139" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="140" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="141" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="142" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="103" spans="1:43" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A103" s="19"/>
+    </row>
+    <row r="104" spans="1:43" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A104" s="19"/>
+    </row>
+    <row r="105" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="106" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="107" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="108" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="109" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="110" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="111" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="112" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="113" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="114" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="115" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="116" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="117" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="118" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="119" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="120" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="121" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="122" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="123" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="124" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="125" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="126" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="127" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="128" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="129" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="130" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="131" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="132" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="133" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="134" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="135" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="136" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="137" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="138" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="139" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="140" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="141" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="142" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="143" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="144" customFormat="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="12">
     <mergeCell ref="A6:A7"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A8:H8"/>
-    <mergeCell ref="A43:H43"/>
-    <mergeCell ref="A58:H58"/>
+    <mergeCell ref="A44:H44"/>
+    <mergeCell ref="A59:H59"/>
     <mergeCell ref="B6:B7"/>
     <mergeCell ref="A5:H5"/>
     <mergeCell ref="G1:H1"/>

</xml_diff>